<commit_message>
2289 - Use generic headings in assessment template
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/_99_publication/monthly_tracker_filled_posts/templates/assessment_template.xlsx
+++ b/projects/_99_publication/monthly_tracker_filled_posts/templates/assessment_template.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="38">
   <si>
     <t>Monthly tracking updates</t>
   </si>
@@ -77,7 +77,7 @@
     <t>Monthly filled posts estimates</t>
   </si>
   <si>
-    <t>% change since end of March</t>
+    <t>Cumulative % change</t>
   </si>
   <si>
     <t>Monthly CQC locations</t>
@@ -144,6 +144,12 @@
   </si>
   <si>
     <t>Skills for Care makes an estimate for all locations, however some may not have submitted to the Capacity Tracker.</t>
+  </si>
+  <si>
+    <t>Comparison of Skills for Care's estimate of filled posts to Capacity Tracker - Since July 2021 (quarterly)</t>
+  </si>
+  <si>
+    <t>- Must have a Capacity Tracker figure in all months from end of July 2021 onwards.</t>
   </si>
 </sst>
 </file>
@@ -23852,13 +23858,17 @@
         <v>1</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="13"/>
+      <c r="E27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="F27" s="14"/>
       <c r="L27" s="13" t="s">
         <v>1</v>
       </c>
       <c r="M27" s="14"/>
-      <c r="N27" s="13"/>
+      <c r="N27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="O27" s="14"/>
       <c r="U27" s="8"/>
       <c r="V27" s="8"/>
@@ -24429,13 +24439,17 @@
         <v>1</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="13"/>
+      <c r="E27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="F27" s="14"/>
       <c r="L27" s="13" t="s">
         <v>1</v>
       </c>
       <c r="M27" s="14"/>
-      <c r="N27" s="13"/>
+      <c r="N27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="O27" s="14"/>
       <c r="P27" s="8"/>
       <c r="Q27" s="7"/>
@@ -25076,7 +25090,9 @@
     </row>
     <row r="4" spans="2:21" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="2:21" ht="18" x14ac:dyDescent="0.25">
-      <c r="B7" s="30"/>
+      <c r="B7" s="30" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="9" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
@@ -25146,7 +25162,9 @@
       <c r="U13" s="7"/>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B14" s="54"/>
+      <c r="B14" s="54" t="s">
+        <v>37</v>
+      </c>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
       <c r="E14" s="48"/>
@@ -25284,13 +25302,17 @@
         <v>1</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="13"/>
+      <c r="E27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="F27" s="14"/>
       <c r="L27" s="13" t="s">
         <v>1</v>
       </c>
       <c r="M27" s="14"/>
-      <c r="N27" s="13"/>
+      <c r="N27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="O27" s="14"/>
       <c r="P27" s="8"/>
       <c r="Q27" s="7"/>
@@ -26081,7 +26103,9 @@
     </row>
     <row r="4" spans="2:21" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="2:21" ht="18" x14ac:dyDescent="0.25">
-      <c r="B7" s="30"/>
+      <c r="B7" s="30" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="9" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
@@ -26288,7 +26312,9 @@
         <v>1</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="13"/>
+      <c r="E27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="F27" s="14"/>
       <c r="G27" s="37" t="s">
         <v>23</v>
@@ -26297,7 +26323,9 @@
         <v>1</v>
       </c>
       <c r="M27" s="14"/>
-      <c r="N27" s="13"/>
+      <c r="N27" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="O27" s="14"/>
       <c r="P27" s="37" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
2289 - Revert B7 and B14 template text changes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/_99_publication/monthly_tracker_filled_posts/templates/assessment_template.xlsx
+++ b/projects/_99_publication/monthly_tracker_filled_posts/templates/assessment_template.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="36">
   <si>
     <t>Monthly tracking updates</t>
   </si>
@@ -144,12 +144,6 @@
   </si>
   <si>
     <t>Skills for Care makes an estimate for all locations, however some may not have submitted to the Capacity Tracker.</t>
-  </si>
-  <si>
-    <t>Comparison of Skills for Care's estimate of filled posts to Capacity Tracker - Since July 2021 (quarterly)</t>
-  </si>
-  <si>
-    <t>- Must have a Capacity Tracker figure in all months from end of July 2021 onwards.</t>
   </si>
 </sst>
 </file>
@@ -25090,9 +25084,7 @@
     </row>
     <row r="4" spans="2:21" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="2:21" ht="18" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
-        <v>36</v>
-      </c>
+      <c r="B7" s="30"/>
     </row>
     <row r="9" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
@@ -25162,9 +25154,7 @@
       <c r="U13" s="7"/>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B14" s="54" t="s">
-        <v>37</v>
-      </c>
+      <c r="B14" s="54"/>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
       <c r="E14" s="48"/>
@@ -26103,9 +26093,7 @@
     </row>
     <row r="4" spans="2:21" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="2:21" ht="18" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
-        <v>36</v>
-      </c>
+      <c r="B7" s="30"/>
     </row>
     <row r="9" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">

</xml_diff>

<commit_message>
2318 - Replace assessment heading literals with column values
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/_99_publication/monthly_tracker_filled_posts/templates/assessment_template.xlsx
+++ b/projects/_99_publication/monthly_tracker_filled_posts/templates/assessment_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
-  <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC569A31-188A-4187-B9E5-78F342640612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578AEFDC-B8C3-4B04-B070-B8218443EF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="779" xr2:uid="{E876E9E8-942E-455D-9B41-2B7C7CFBA90D}"/>
   </bookViews>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>CQC care home with nursing</t>
-  </si>
-  <si>
-    <t>CQC care home without nursing</t>
   </si>
   <si>
     <t>CQC non-residential</t>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>Skills for Care makes an estimate for all locations, however some may not have submitted to the Capacity Tracker.</t>
+  </si>
+  <si>
+    <t>CQC care only home</t>
   </si>
 </sst>
 </file>
@@ -19501,7 +19501,7 @@
     </row>
     <row r="9" spans="2:41" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -19572,7 +19572,7 @@
     </row>
     <row r="11" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B11" s="54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -19613,7 +19613,7 @@
     </row>
     <row r="12" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B12" s="54" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -19654,7 +19654,7 @@
     </row>
     <row r="13" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B13" s="54" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -19695,7 +19695,7 @@
     </row>
     <row r="14" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B14" s="54" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
@@ -19960,10 +19960,10 @@
         <v>7</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J23" s="20" t="s">
         <v>5</v>
@@ -19975,10 +19975,10 @@
         <v>7</v>
       </c>
       <c r="M23" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P23" s="6"/>
       <c r="Q23" s="8"/>
@@ -20461,7 +20461,7 @@
     </row>
     <row r="40" spans="2:36" s="33" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B40" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
@@ -20494,7 +20494,7 @@
     <row r="42" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B42" s="1"/>
       <c r="C42" s="22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D42" s="23"/>
       <c r="E42" s="23"/>
@@ -20522,10 +20522,10 @@
         <v>7</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="G43" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -20539,10 +20539,10 @@
         <v>7</v>
       </c>
       <c r="M43" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="N43" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" spans="2:36" s="33" customFormat="1" x14ac:dyDescent="0.2">
@@ -20816,7 +20816,7 @@
     <row r="60" spans="2:36" s="33" customFormat="1" ht="14.25" x14ac:dyDescent="0.2"/>
     <row r="61" spans="2:36" s="33" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" spans="2:36" s="33" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
@@ -20838,7 +20838,7 @@
       <c r="G63" s="23"/>
       <c r="H63" s="8"/>
       <c r="J63" s="22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K63" s="23"/>
       <c r="L63" s="23"/>
@@ -20864,10 +20864,10 @@
         <v>7</v>
       </c>
       <c r="F64" s="47" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="G64" s="47" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I64" s="2"/>
       <c r="J64" s="46" t="s">
@@ -20880,10 +20880,10 @@
         <v>7</v>
       </c>
       <c r="M64" s="47" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="N64" s="47" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="8"/>
@@ -21260,7 +21260,7 @@
     </row>
     <row r="80" spans="2:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B80" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="6"/>
@@ -21274,7 +21274,7 @@
     </row>
     <row r="82" spans="2:34" x14ac:dyDescent="0.2">
       <c r="C82" s="22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D82" s="23"/>
       <c r="E82" s="23"/>
@@ -21282,7 +21282,7 @@
       <c r="G82" s="23"/>
       <c r="H82" s="8"/>
       <c r="J82" s="22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K82" s="23"/>
       <c r="L82" s="23"/>
@@ -21301,10 +21301,10 @@
         <v>7</v>
       </c>
       <c r="F83" s="47" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="G83" s="47" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I83" s="2"/>
       <c r="J83" s="46" t="s">
@@ -21317,10 +21317,10 @@
         <v>7</v>
       </c>
       <c r="M83" s="47" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="N83" s="47" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="84" spans="2:34" x14ac:dyDescent="0.2">
@@ -21959,7 +21959,7 @@
     <row r="4" spans="2:41" s="2" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="2:41" ht="18" x14ac:dyDescent="0.25">
       <c r="B7" s="30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -21984,7 +21984,7 @@
     </row>
     <row r="9" spans="2:41" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -22055,7 +22055,7 @@
     </row>
     <row r="11" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B11" s="54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -22096,7 +22096,7 @@
     </row>
     <row r="12" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B12" s="54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -22137,7 +22137,7 @@
     </row>
     <row r="13" spans="2:41" x14ac:dyDescent="0.2">
       <c r="B13" s="54" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -22337,7 +22337,7 @@
     </row>
     <row r="20" spans="2:41" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="2:41" x14ac:dyDescent="0.2">
@@ -22360,10 +22360,10 @@
         <v>7</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S22" s="6"/>
       <c r="T22" s="8"/>
@@ -22792,7 +22792,7 @@
     </row>
     <row r="61" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S61" s="6"/>
     </row>
@@ -22810,10 +22810,10 @@
         <v>7</v>
       </c>
       <c r="G63" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="H63" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64" spans="2:19" x14ac:dyDescent="0.2">
@@ -23239,7 +23239,7 @@
     </row>
     <row r="103" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B103" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="105" spans="2:19" ht="45" x14ac:dyDescent="0.2">
@@ -23254,10 +23254,10 @@
         <v>7</v>
       </c>
       <c r="G105" s="17" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="H105" s="17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="106" spans="2:19" x14ac:dyDescent="0.2">
@@ -23559,6 +23559,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>
 </file>
 
@@ -23589,7 +23590,7 @@
     </row>
     <row r="9" spans="2:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -23617,7 +23618,7 @@
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B11" s="54" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -23663,7 +23664,7 @@
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B13" s="54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -23709,7 +23710,7 @@
     </row>
     <row r="15" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B15" s="54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -23806,7 +23807,7 @@
         <v>6</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U23" s="8"/>
       <c r="V23" s="8"/>
@@ -23825,11 +23826,11 @@
     </row>
     <row r="25" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" s="8"/>
       <c r="K25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M25" s="8"/>
       <c r="U25" s="8"/>
@@ -23853,7 +23854,7 @@
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F27" s="14"/>
       <c r="L27" s="13" t="s">
@@ -23861,7 +23862,7 @@
       </c>
       <c r="M27" s="14"/>
       <c r="N27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O27" s="14"/>
       <c r="U27" s="8"/>
@@ -23873,28 +23874,28 @@
     </row>
     <row r="28" spans="2:26" ht="30" x14ac:dyDescent="0.2">
       <c r="C28" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>21</v>
+      <c r="E28" s="20" t="s">
+        <v>19</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="F28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="17" t="s">
-        <v>21</v>
+      <c r="L28" s="20" t="s">
+        <v>19</v>
       </c>
-      <c r="L28" s="20" t="s">
+      <c r="M28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M28" s="17" t="s">
-        <v>21</v>
-      </c>
       <c r="N28" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O28" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="U28" s="8"/>
       <c r="V28" s="8"/>
@@ -24085,7 +24086,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -24116,7 +24118,7 @@
     </row>
     <row r="9" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -24142,7 +24144,7 @@
     </row>
     <row r="11" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B11" s="54" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -24186,7 +24188,7 @@
     </row>
     <row r="13" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B13" s="54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -24232,7 +24234,7 @@
     </row>
     <row r="15" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B15" s="54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -24367,7 +24369,7 @@
         <v>6</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P23" s="8"/>
       <c r="Q23" s="7"/>
@@ -24396,11 +24398,11 @@
     </row>
     <row r="25" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" s="8"/>
       <c r="K25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M25" s="8"/>
       <c r="P25" s="8"/>
@@ -24434,7 +24436,7 @@
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F27" s="14"/>
       <c r="L27" s="13" t="s">
@@ -24442,7 +24444,7 @@
       </c>
       <c r="M27" s="14"/>
       <c r="N27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O27" s="14"/>
       <c r="P27" s="8"/>
@@ -24459,28 +24461,28 @@
     </row>
     <row r="28" spans="2:28" ht="30" x14ac:dyDescent="0.2">
       <c r="C28" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>21</v>
+      <c r="E28" s="20" t="s">
+        <v>19</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="F28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="17" t="s">
-        <v>21</v>
+      <c r="L28" s="20" t="s">
+        <v>19</v>
       </c>
-      <c r="L28" s="20" t="s">
+      <c r="M28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M28" s="17" t="s">
-        <v>21</v>
-      </c>
       <c r="N28" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O28" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P28" s="8"/>
       <c r="Q28" s="7"/>
@@ -25056,7 +25058,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -25088,7 +25091,7 @@
     </row>
     <row r="9" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -25108,7 +25111,7 @@
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B11" s="54" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -25138,7 +25141,7 @@
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B13" s="54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -25170,7 +25173,7 @@
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B15" s="54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -25250,7 +25253,7 @@
         <v>6</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P23" s="8"/>
       <c r="Q23" s="7"/>
@@ -25267,11 +25270,11 @@
     </row>
     <row r="25" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" s="8"/>
       <c r="K25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M25" s="8"/>
       <c r="P25" s="8"/>
@@ -25293,7 +25296,7 @@
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F27" s="14"/>
       <c r="L27" s="13" t="s">
@@ -25301,7 +25304,7 @@
       </c>
       <c r="M27" s="14"/>
       <c r="N27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O27" s="14"/>
       <c r="P27" s="8"/>
@@ -25312,28 +25315,28 @@
     </row>
     <row r="28" spans="2:23" ht="30" x14ac:dyDescent="0.2">
       <c r="C28" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>21</v>
+      <c r="E28" s="20" t="s">
+        <v>19</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="F28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="F28" s="17" t="s">
-        <v>21</v>
+      <c r="L28" s="20" t="s">
+        <v>19</v>
       </c>
-      <c r="L28" s="20" t="s">
+      <c r="M28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M28" s="17" t="s">
-        <v>21</v>
-      </c>
       <c r="N28" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O28" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P28" s="8"/>
       <c r="Q28" s="7"/>
@@ -26065,7 +26068,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -26097,7 +26101,7 @@
     </row>
     <row r="9" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -26119,7 +26123,7 @@
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B11" s="54" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -26151,7 +26155,7 @@
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B13" s="54" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -26169,7 +26173,7 @@
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B14" s="54" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
@@ -26258,7 +26262,7 @@
         <v>6</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P23" s="8"/>
       <c r="Q23" s="7"/>
@@ -26273,16 +26277,16 @@
     </row>
     <row r="25" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M25" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P25" s="8"/>
       <c r="Q25" s="7"/>
@@ -26301,22 +26305,22 @@
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F27" s="14"/>
       <c r="G27" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L27" s="13" t="s">
         <v>1</v>
       </c>
       <c r="M27" s="14"/>
       <c r="N27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O27" s="14"/>
       <c r="P27" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q27" s="7"/>
       <c r="T27" s="8"/>
@@ -26324,29 +26328,29 @@
     </row>
     <row r="28" spans="2:21" ht="30" x14ac:dyDescent="0.2">
       <c r="C28" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>21</v>
-      </c>
       <c r="E28" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G28" s="38"/>
       <c r="L28" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="M28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M28" s="17" t="s">
-        <v>21</v>
-      </c>
       <c r="N28" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O28" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P28" s="39"/>
       <c r="Q28" s="7"/>
@@ -26934,6 +26938,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>